<commit_message>
Fix over-cleaned BSX/WMB in as_of=6/10 snapshot + regen 6/10-6/11 risk reports
The earlier zombie cleanup removed BSX/WMB from inventory_mrpt_20260617
(as_of=6/10), but BSX/WMB was legitimately active on 6/10 (closed 6/11).
Restored it from the correct 20260612_031919 snapshot.

6/10 PnL-vs-Risk diff improved: +$2,705 → +$777 (OK).

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/trading_signals/risk_management/risk_workbook_20260611_031025.xlsx
+++ b/trading_signals/risk_management/risk_workbook_20260611_031025.xlsx
@@ -231,7 +231,7 @@
     <xf numFmtId="0" fontId="4" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="4" fontId="8" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="4" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
@@ -731,7 +731,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Signal date 2026-06-10  ·  Generated 2026-06-25T01:49:33  ·  Scope: MRPT+MTFS pairs book (model-based, broker-reconciled)</t>
+          <t>Signal date 2026-06-10  ·  Generated 2026-06-25T02:04:51  ·  Scope: MRPT+MTFS pairs book (model-based, broker-reconciled)</t>
         </is>
       </c>
     </row>
@@ -752,7 +752,7 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>1.243</v>
+        <v>1.409</v>
       </c>
     </row>
     <row r="6">
@@ -762,7 +762,7 @@
         </is>
       </c>
       <c r="B6" s="6" t="n">
-        <v>0.406</v>
+        <v>0.405</v>
       </c>
     </row>
     <row r="7">
@@ -772,7 +772,7 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>0.804</v>
+        <v>0.768</v>
       </c>
     </row>
     <row r="8">
@@ -782,7 +782,7 @@
         </is>
       </c>
       <c r="B8" s="4" t="n">
-        <v>21466.42</v>
+        <v>21654.02</v>
       </c>
     </row>
     <row r="9">
@@ -792,7 +792,7 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>2.04</v>
+        <v>2.05</v>
       </c>
     </row>
     <row r="10">
@@ -802,7 +802,7 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>19.64</v>
+        <v>19.82</v>
       </c>
     </row>
     <row r="11">
@@ -854,7 +854,7 @@
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>1.243</v>
+        <v>1.409</v>
       </c>
     </row>
     <row r="16">
@@ -876,7 +876,7 @@
         </is>
       </c>
       <c r="B17" s="5" t="n">
-        <v>33.32</v>
+        <v>29.41</v>
       </c>
     </row>
     <row r="18">
@@ -886,7 +886,7 @@
         </is>
       </c>
       <c r="B18" s="5" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="19">
@@ -896,7 +896,7 @@
         </is>
       </c>
       <c r="B19" s="5" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="20">
@@ -925,7 +925,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D20"/>
+  <dimension ref="A1:D21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -947,7 +947,7 @@
         </is>
       </c>
       <c r="B3" s="4" t="n">
-        <v>21466.42</v>
+        <v>21654.02</v>
       </c>
     </row>
     <row r="4">
@@ -957,7 +957,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>30353.13</v>
+        <v>30618.39</v>
       </c>
     </row>
     <row r="5">
@@ -967,7 +967,7 @@
         </is>
       </c>
       <c r="B5" s="4" t="n">
-        <v>207154.36</v>
+        <v>208964.68</v>
       </c>
     </row>
     <row r="6">
@@ -977,7 +977,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>19.64</v>
+        <v>19.82</v>
       </c>
     </row>
     <row r="7">
@@ -987,7 +987,7 @@
         </is>
       </c>
       <c r="B7" s="4" t="n">
-        <v>13540.83</v>
+        <v>12921.92</v>
       </c>
     </row>
     <row r="8">
@@ -997,7 +997,7 @@
         </is>
       </c>
       <c r="B8" s="4" t="n">
-        <v>20936.62</v>
+        <v>20091.21</v>
       </c>
     </row>
     <row r="10">
@@ -1031,10 +1031,10 @@
         </is>
       </c>
       <c r="B12" s="4" t="n">
-        <v>5751.57</v>
+        <v>5283.66</v>
       </c>
       <c r="C12" s="7" t="n">
-        <v>26.79</v>
+        <v>24.4</v>
       </c>
     </row>
     <row r="13">
@@ -1044,10 +1044,10 @@
         </is>
       </c>
       <c r="B13" s="13" t="n">
-        <v>5031.28</v>
+        <v>4929.31</v>
       </c>
       <c r="C13" s="17" t="n">
-        <v>23.44</v>
+        <v>22.76</v>
       </c>
     </row>
     <row r="14">
@@ -1057,10 +1057,10 @@
         </is>
       </c>
       <c r="B14" s="4" t="n">
-        <v>3513.61</v>
+        <v>3441.71</v>
       </c>
       <c r="C14" s="7" t="n">
-        <v>16.37</v>
+        <v>15.89</v>
       </c>
     </row>
     <row r="15">
@@ -1070,10 +1070,10 @@
         </is>
       </c>
       <c r="B15" s="13" t="n">
-        <v>2357.17</v>
+        <v>2504.17</v>
       </c>
       <c r="C15" s="17" t="n">
-        <v>10.98</v>
+        <v>11.56</v>
       </c>
     </row>
     <row r="16">
@@ -1083,10 +1083,10 @@
         </is>
       </c>
       <c r="B16" s="4" t="n">
-        <v>1748.73</v>
+        <v>1804.75</v>
       </c>
       <c r="C16" s="7" t="n">
-        <v>8.15</v>
+        <v>8.33</v>
       </c>
     </row>
     <row r="17">
@@ -1096,36 +1096,36 @@
         </is>
       </c>
       <c r="B17" s="13" t="n">
-        <v>1692.05</v>
+        <v>1616.46</v>
       </c>
       <c r="C17" s="17" t="n">
-        <v>7.88</v>
+        <v>7.46</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="10" t="inlineStr">
         <is>
-          <t>HST/MOS</t>
+          <t>BSX/WMB</t>
         </is>
       </c>
       <c r="B18" s="4" t="n">
-        <v>783.95</v>
+        <v>774.73</v>
       </c>
       <c r="C18" s="7" t="n">
-        <v>3.65</v>
+        <v>3.58</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="12" t="inlineStr">
         <is>
-          <t>HAS/PFE</t>
+          <t>HST/MOS</t>
         </is>
       </c>
       <c r="B19" s="13" t="n">
-        <v>309.26</v>
+        <v>728.67</v>
       </c>
       <c r="C19" s="17" t="n">
-        <v>1.44</v>
+        <v>3.37</v>
       </c>
     </row>
     <row r="20">
@@ -1135,10 +1135,23 @@
         </is>
       </c>
       <c r="B20" s="4" t="n">
-        <v>278.81</v>
+        <v>314.67</v>
       </c>
       <c r="C20" s="7" t="n">
-        <v>1.3</v>
+        <v>1.45</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="12" t="inlineStr">
+        <is>
+          <t>HAS/PFE</t>
+        </is>
+      </c>
+      <c r="B21" s="13" t="n">
+        <v>255.89</v>
+      </c>
+      <c r="C21" s="17" t="n">
+        <v>1.18</v>
       </c>
     </row>
   </sheetData>
@@ -1272,19 +1285,19 @@
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
         <is>
-          <t>KLAC</t>
+          <t>BSX</t>
         </is>
       </c>
       <c r="B9" s="17" t="inlineStr">
         <is>
-          <t>KLAC/REGN</t>
+          <t>BSX/WMB</t>
         </is>
       </c>
       <c r="C9" s="13" t="n">
-        <v>670</v>
+        <v>1817</v>
       </c>
       <c r="D9" s="13" t="n">
-        <v>3046345</v>
+        <v>18762823</v>
       </c>
       <c r="E9" s="17" t="n">
         <v>0</v>
@@ -1293,19 +1306,19 @@
     <row r="10">
       <c r="A10" s="10" t="inlineStr">
         <is>
-          <t>REGN</t>
+          <t>WMB</t>
         </is>
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>KLAC/REGN</t>
-        </is>
-      </c>
-      <c r="C10" s="11" t="n">
-        <v>23</v>
+          <t>BSX/WMB</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="n">
+        <v>1195</v>
       </c>
       <c r="D10" s="4" t="n">
-        <v>1102391</v>
+        <v>6192571</v>
       </c>
       <c r="E10" s="7" t="n">
         <v>0</v>
@@ -1314,19 +1327,19 @@
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
         <is>
-          <t>NUE</t>
+          <t>KLAC</t>
         </is>
       </c>
       <c r="B11" s="17" t="inlineStr">
         <is>
-          <t>NUE/INTU</t>
+          <t>KLAC/REGN</t>
         </is>
       </c>
       <c r="C11" s="13" t="n">
-        <v>329</v>
+        <v>670</v>
       </c>
       <c r="D11" s="13" t="n">
-        <v>1408637</v>
+        <v>3046345</v>
       </c>
       <c r="E11" s="17" t="n">
         <v>0</v>
@@ -1335,19 +1348,19 @@
     <row r="12">
       <c r="A12" s="10" t="inlineStr">
         <is>
-          <t>INTU</t>
+          <t>REGN</t>
         </is>
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>NUE/INTU</t>
+          <t>KLAC/REGN</t>
         </is>
       </c>
       <c r="C12" s="11" t="n">
-        <v>82</v>
+        <v>23</v>
       </c>
       <c r="D12" s="4" t="n">
-        <v>6155217</v>
+        <v>1102391</v>
       </c>
       <c r="E12" s="7" t="n">
         <v>0</v>
@@ -1361,7 +1374,7 @@
       </c>
       <c r="B13" s="17" t="inlineStr">
         <is>
-          <t>NUE/MKTX</t>
+          <t>NUE/INTU</t>
         </is>
       </c>
       <c r="C13" s="13" t="n">
@@ -1377,19 +1390,19 @@
     <row r="14">
       <c r="A14" s="10" t="inlineStr">
         <is>
-          <t>MKTX</t>
+          <t>INTU</t>
         </is>
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>NUE/MKTX</t>
-        </is>
-      </c>
-      <c r="C14" s="4" t="n">
-        <v>422</v>
+          <t>NUE/INTU</t>
+        </is>
+      </c>
+      <c r="C14" s="11" t="n">
+        <v>82</v>
       </c>
       <c r="D14" s="4" t="n">
-        <v>721296</v>
+        <v>6155217</v>
       </c>
       <c r="E14" s="7" t="n">
         <v>0</v>
@@ -1398,19 +1411,19 @@
     <row r="15">
       <c r="A15" s="12" t="inlineStr">
         <is>
-          <t>STLD</t>
+          <t>NUE</t>
         </is>
       </c>
       <c r="B15" s="17" t="inlineStr">
         <is>
-          <t>STLD/UHS</t>
+          <t>NUE/MKTX</t>
         </is>
       </c>
       <c r="C15" s="13" t="n">
-        <v>386</v>
+        <v>329</v>
       </c>
       <c r="D15" s="13" t="n">
-        <v>1103538</v>
+        <v>1408637</v>
       </c>
       <c r="E15" s="17" t="n">
         <v>0</v>
@@ -1419,19 +1432,19 @@
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>UHS</t>
+          <t>MKTX</t>
         </is>
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>STLD/UHS</t>
+          <t>NUE/MKTX</t>
         </is>
       </c>
       <c r="C16" s="4" t="n">
-        <v>358</v>
+        <v>422</v>
       </c>
       <c r="D16" s="4" t="n">
-        <v>1031090</v>
+        <v>721296</v>
       </c>
       <c r="E16" s="7" t="n">
         <v>0</v>
@@ -1445,11 +1458,11 @@
       </c>
       <c r="B17" s="17" t="inlineStr">
         <is>
-          <t>STLD/FMC</t>
+          <t>STLD/UHS</t>
         </is>
       </c>
       <c r="C17" s="13" t="n">
-        <v>628</v>
+        <v>386</v>
       </c>
       <c r="D17" s="13" t="n">
         <v>1103538</v>
@@ -1461,19 +1474,19 @@
     <row r="18">
       <c r="A18" s="10" t="inlineStr">
         <is>
-          <t>HST</t>
+          <t>UHS</t>
         </is>
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>HST/MOS</t>
+          <t>STLD/UHS</t>
         </is>
       </c>
       <c r="C18" s="4" t="n">
-        <v>2247</v>
+        <v>358</v>
       </c>
       <c r="D18" s="4" t="n">
-        <v>8680193</v>
+        <v>1031090</v>
       </c>
       <c r="E18" s="7" t="n">
         <v>0</v>
@@ -1482,19 +1495,19 @@
     <row r="19">
       <c r="A19" s="12" t="inlineStr">
         <is>
-          <t>MOS</t>
+          <t>STLD</t>
         </is>
       </c>
       <c r="B19" s="17" t="inlineStr">
         <is>
-          <t>HST/MOS</t>
+          <t>STLD/FMC</t>
         </is>
       </c>
       <c r="C19" s="13" t="n">
-        <v>2168</v>
+        <v>628</v>
       </c>
       <c r="D19" s="13" t="n">
-        <v>8809289</v>
+        <v>1103538</v>
       </c>
       <c r="E19" s="17" t="n">
         <v>0</v>
@@ -1503,19 +1516,19 @@
     <row r="20">
       <c r="A20" s="10" t="inlineStr">
         <is>
-          <t>KLAC</t>
+          <t>HST</t>
         </is>
       </c>
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>KLAC/TRMB</t>
+          <t>HST/MOS</t>
         </is>
       </c>
       <c r="C20" s="4" t="n">
-        <v>470</v>
+        <v>2247</v>
       </c>
       <c r="D20" s="4" t="n">
-        <v>3046345</v>
+        <v>8680193</v>
       </c>
       <c r="E20" s="7" t="n">
         <v>0</v>
@@ -1574,10 +1587,10 @@
         </is>
       </c>
       <c r="B4" s="19" t="n">
-        <v>-42392.8</v>
+        <v>-40494.62</v>
       </c>
       <c r="C4" s="22" t="n">
-        <v>-4.02</v>
+        <v>-3.84</v>
       </c>
     </row>
     <row r="5">
@@ -1587,10 +1600,10 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>-84785.60000000001</v>
+        <v>-80989.23</v>
       </c>
       <c r="C5" s="20" t="n">
-        <v>-8.039999999999999</v>
+        <v>-7.68</v>
       </c>
     </row>
     <row r="6">
@@ -1600,10 +1613,10 @@
         </is>
       </c>
       <c r="B6" s="19" t="n">
-        <v>-42392.8</v>
+        <v>-40494.62</v>
       </c>
       <c r="C6" s="22" t="n">
-        <v>-4.02</v>
+        <v>-3.84</v>
       </c>
     </row>
     <row r="7">
@@ -1695,7 +1708,7 @@
         </is>
       </c>
       <c r="C4" s="30" t="n">
-        <v>0.3</v>
+        <v>0.61</v>
       </c>
       <c r="D4" s="30" t="n">
         <v>3</v>
@@ -1721,7 +1734,7 @@
         </is>
       </c>
       <c r="C5" s="30" t="n">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="D5" s="30" t="n">
         <v>0.5</v>
@@ -1866,28 +1879,28 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="31" t="inlineStr">
+      <c r="A11" s="29" t="inlineStr">
         <is>
           <t>sector_net</t>
         </is>
       </c>
-      <c r="B11" s="32" t="inlineStr">
+      <c r="B11" s="30" t="inlineStr">
         <is>
           <t>materials</t>
         </is>
       </c>
-      <c r="C11" s="32" t="n">
-        <v>33.32</v>
-      </c>
-      <c r="D11" s="32" t="n">
+      <c r="C11" s="30" t="n">
+        <v>29.41</v>
+      </c>
+      <c r="D11" s="30" t="n">
         <v>30</v>
       </c>
-      <c r="E11" s="32" t="n">
+      <c r="E11" s="30" t="n">
         <v>50</v>
       </c>
-      <c r="F11" s="32" t="inlineStr">
-        <is>
-          <t>amber</t>
+      <c r="F11" s="30" t="inlineStr">
+        <is>
+          <t>green</t>
         </is>
       </c>
     </row>
@@ -1903,7 +1916,7 @@
         </is>
       </c>
       <c r="C12" s="30" t="n">
-        <v>18.49</v>
+        <v>16.32</v>
       </c>
       <c r="D12" s="30" t="n">
         <v>20</v>
@@ -1929,7 +1942,7 @@
         </is>
       </c>
       <c r="C13" s="34" t="n">
-        <v>0.8</v>
+        <v>0.77</v>
       </c>
       <c r="D13" s="34" t="n">
         <v>0.3</v>
@@ -1955,7 +1968,7 @@
         </is>
       </c>
       <c r="C14" s="30" t="n">
-        <v>2.04</v>
+        <v>2.05</v>
       </c>
       <c r="D14" s="30" t="n">
         <v>3</v>
@@ -1981,7 +1994,7 @@
         </is>
       </c>
       <c r="C15" s="30" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D15" s="30" t="n">
         <v>8</v>
@@ -2031,7 +2044,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J21"/>
+  <dimension ref="A1:J23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2196,36 +2209,36 @@
     <row r="6">
       <c r="A6" s="12" t="inlineStr">
         <is>
-          <t>MTFS</t>
+          <t>MRPT</t>
         </is>
       </c>
       <c r="B6" s="17" t="inlineStr">
         <is>
-          <t>KLAC/REGN</t>
+          <t>BSX/WMB</t>
         </is>
       </c>
       <c r="C6" s="17" t="inlineStr">
         <is>
-          <t>KLAC</t>
+          <t>BSX</t>
         </is>
       </c>
       <c r="D6" s="17" t="inlineStr">
         <is>
-          <t>long</t>
+          <t>short</t>
         </is>
       </c>
       <c r="E6" s="26" t="n">
-        <v>670</v>
-      </c>
-      <c r="F6" s="13" t="n">
-        <v>213.56</v>
-      </c>
-      <c r="G6" s="13" t="n">
-        <v>143087.88</v>
+        <v>-1817</v>
+      </c>
+      <c r="F6" s="15" t="n">
+        <v>48.34</v>
+      </c>
+      <c r="G6" s="18" t="n">
+        <v>-87833.78</v>
       </c>
       <c r="H6" s="17" t="inlineStr">
         <is>
-          <t>tech</t>
+          <t>health</t>
         </is>
       </c>
       <c r="I6" s="17" t="n">
@@ -2233,43 +2246,43 @@
       </c>
       <c r="J6" s="17" t="inlineStr">
         <is>
-          <t>beta_neutral_long_term</t>
+          <t>tight_stop</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="10" t="inlineStr">
         <is>
-          <t>MTFS</t>
+          <t>MRPT</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>KLAC/REGN</t>
+          <t>BSX/WMB</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>REGN</t>
+          <t>WMB</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>long</t>
         </is>
       </c>
       <c r="E7" s="24" t="n">
-        <v>-23</v>
-      </c>
-      <c r="F7" s="4" t="n">
-        <v>601.65</v>
-      </c>
-      <c r="G7" s="19" t="n">
-        <v>-13837.95</v>
+        <v>1195</v>
+      </c>
+      <c r="F7" s="11" t="n">
+        <v>72.26000000000001</v>
+      </c>
+      <c r="G7" s="4" t="n">
+        <v>86350.7</v>
       </c>
       <c r="H7" s="7" t="inlineStr">
         <is>
-          <t>health</t>
+          <t>energy</t>
         </is>
       </c>
       <c r="I7" s="7" t="n">
@@ -2277,7 +2290,7 @@
       </c>
       <c r="J7" s="7" t="inlineStr">
         <is>
-          <t>beta_neutral_long_term</t>
+          <t>tight_stop</t>
         </is>
       </c>
     </row>
@@ -2289,12 +2302,12 @@
       </c>
       <c r="B8" s="17" t="inlineStr">
         <is>
-          <t>NUE/INTU</t>
+          <t>KLAC/REGN</t>
         </is>
       </c>
       <c r="C8" s="17" t="inlineStr">
         <is>
-          <t>NUE</t>
+          <t>KLAC</t>
         </is>
       </c>
       <c r="D8" s="17" t="inlineStr">
@@ -2303,17 +2316,17 @@
         </is>
       </c>
       <c r="E8" s="26" t="n">
-        <v>329</v>
+        <v>670</v>
       </c>
       <c r="F8" s="13" t="n">
-        <v>250.49</v>
+        <v>213.56</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>82411.21000000001</v>
+        <v>143087.88</v>
       </c>
       <c r="H8" s="17" t="inlineStr">
         <is>
-          <t>materials</t>
+          <t>tech</t>
         </is>
       </c>
       <c r="I8" s="17" t="n">
@@ -2321,7 +2334,7 @@
       </c>
       <c r="J8" s="17" t="inlineStr">
         <is>
-          <t>conservative</t>
+          <t>beta_neutral_long_term</t>
         </is>
       </c>
     </row>
@@ -2333,12 +2346,12 @@
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>NUE/INTU</t>
+          <t>KLAC/REGN</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>INTU</t>
+          <t>REGN</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
@@ -2347,17 +2360,17 @@
         </is>
       </c>
       <c r="E9" s="24" t="n">
-        <v>-82</v>
+        <v>-23</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>284.22</v>
+        <v>601.65</v>
       </c>
       <c r="G9" s="19" t="n">
-        <v>-23306.04</v>
+        <v>-13837.95</v>
       </c>
       <c r="H9" s="7" t="inlineStr">
         <is>
-          <t>tech</t>
+          <t>health</t>
         </is>
       </c>
       <c r="I9" s="7" t="n">
@@ -2365,7 +2378,7 @@
       </c>
       <c r="J9" s="7" t="inlineStr">
         <is>
-          <t>conservative</t>
+          <t>beta_neutral_long_term</t>
         </is>
       </c>
     </row>
@@ -2377,7 +2390,7 @@
       </c>
       <c r="B10" s="17" t="inlineStr">
         <is>
-          <t>NUE/MKTX</t>
+          <t>NUE/INTU</t>
         </is>
       </c>
       <c r="C10" s="17" t="inlineStr">
@@ -2409,7 +2422,7 @@
       </c>
       <c r="J10" s="17" t="inlineStr">
         <is>
-          <t>weekly_aligned_windows</t>
+          <t>conservative</t>
         </is>
       </c>
     </row>
@@ -2421,12 +2434,12 @@
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>NUE/MKTX</t>
+          <t>NUE/INTU</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>MKTX</t>
+          <t>INTU</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
@@ -2435,13 +2448,13 @@
         </is>
       </c>
       <c r="E11" s="24" t="n">
-        <v>-422</v>
+        <v>-82</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>116.11</v>
+        <v>284.22</v>
       </c>
       <c r="G11" s="19" t="n">
-        <v>-48998.42</v>
+        <v>-23306.04</v>
       </c>
       <c r="H11" s="7" t="inlineStr">
         <is>
@@ -2453,7 +2466,7 @@
       </c>
       <c r="J11" s="7" t="inlineStr">
         <is>
-          <t>weekly_aligned_windows</t>
+          <t>conservative</t>
         </is>
       </c>
     </row>
@@ -2465,12 +2478,12 @@
       </c>
       <c r="B12" s="17" t="inlineStr">
         <is>
-          <t>STLD/UHS</t>
+          <t>NUE/MKTX</t>
         </is>
       </c>
       <c r="C12" s="17" t="inlineStr">
         <is>
-          <t>STLD</t>
+          <t>NUE</t>
         </is>
       </c>
       <c r="D12" s="17" t="inlineStr">
@@ -2479,13 +2492,13 @@
         </is>
       </c>
       <c r="E12" s="26" t="n">
-        <v>386</v>
+        <v>329</v>
       </c>
       <c r="F12" s="13" t="n">
-        <v>268.34</v>
+        <v>250.49</v>
       </c>
       <c r="G12" s="13" t="n">
-        <v>103579.24</v>
+        <v>82411.21000000001</v>
       </c>
       <c r="H12" s="17" t="inlineStr">
         <is>
@@ -2493,11 +2506,11 @@
         </is>
       </c>
       <c r="I12" s="17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J12" s="17" t="inlineStr">
         <is>
-          <t>no_reversal_protection</t>
+          <t>weekly_aligned_windows</t>
         </is>
       </c>
     </row>
@@ -2509,12 +2522,12 @@
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>STLD/UHS</t>
+          <t>NUE/MKTX</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>UHS</t>
+          <t>MKTX</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
@@ -2523,25 +2536,25 @@
         </is>
       </c>
       <c r="E13" s="24" t="n">
-        <v>-358</v>
+        <v>-422</v>
       </c>
       <c r="F13" s="4" t="n">
-        <v>144.82</v>
+        <v>116.11</v>
       </c>
       <c r="G13" s="19" t="n">
-        <v>-51845.56</v>
+        <v>-48998.42</v>
       </c>
       <c r="H13" s="7" t="inlineStr">
         <is>
-          <t>health</t>
+          <t>tech</t>
         </is>
       </c>
       <c r="I13" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J13" s="7" t="inlineStr">
         <is>
-          <t>no_reversal_protection</t>
+          <t>weekly_aligned_windows</t>
         </is>
       </c>
     </row>
@@ -2553,7 +2566,7 @@
       </c>
       <c r="B14" s="17" t="inlineStr">
         <is>
-          <t>STLD/FMC</t>
+          <t>STLD/UHS</t>
         </is>
       </c>
       <c r="C14" s="17" t="inlineStr">
@@ -2567,13 +2580,13 @@
         </is>
       </c>
       <c r="E14" s="26" t="n">
-        <v>628</v>
+        <v>386</v>
       </c>
       <c r="F14" s="13" t="n">
         <v>268.34</v>
       </c>
       <c r="G14" s="13" t="n">
-        <v>168517.52</v>
+        <v>103579.24</v>
       </c>
       <c r="H14" s="17" t="inlineStr">
         <is>
@@ -2585,7 +2598,7 @@
       </c>
       <c r="J14" s="17" t="inlineStr">
         <is>
-          <t>aggressive</t>
+          <t>no_reversal_protection</t>
         </is>
       </c>
     </row>
@@ -2597,12 +2610,12 @@
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>STLD/FMC</t>
+          <t>STLD/UHS</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>FMC</t>
+          <t>UHS</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
@@ -2611,17 +2624,17 @@
         </is>
       </c>
       <c r="E15" s="24" t="n">
-        <v>-6843</v>
-      </c>
-      <c r="F15" s="11" t="n">
-        <v>10.8</v>
+        <v>-358</v>
+      </c>
+      <c r="F15" s="4" t="n">
+        <v>144.82</v>
       </c>
       <c r="G15" s="19" t="n">
-        <v>-73904.39999999999</v>
+        <v>-51845.56</v>
       </c>
       <c r="H15" s="7" t="inlineStr">
         <is>
-          <t>food</t>
+          <t>health</t>
         </is>
       </c>
       <c r="I15" s="7" t="n">
@@ -2629,7 +2642,7 @@
       </c>
       <c r="J15" s="7" t="inlineStr">
         <is>
-          <t>aggressive</t>
+          <t>no_reversal_protection</t>
         </is>
       </c>
     </row>
@@ -2641,12 +2654,12 @@
       </c>
       <c r="B16" s="17" t="inlineStr">
         <is>
-          <t>HST/MOS</t>
+          <t>STLD/FMC</t>
         </is>
       </c>
       <c r="C16" s="17" t="inlineStr">
         <is>
-          <t>HST</t>
+          <t>STLD</t>
         </is>
       </c>
       <c r="D16" s="17" t="inlineStr">
@@ -2655,25 +2668,25 @@
         </is>
       </c>
       <c r="E16" s="26" t="n">
-        <v>2247</v>
-      </c>
-      <c r="F16" s="15" t="n">
-        <v>23.95</v>
+        <v>628</v>
+      </c>
+      <c r="F16" s="13" t="n">
+        <v>268.34</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>53815.65</v>
+        <v>168517.52</v>
       </c>
       <c r="H16" s="17" t="inlineStr">
         <is>
-          <t>realestate</t>
+          <t>materials</t>
         </is>
       </c>
       <c r="I16" s="17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J16" s="17" t="inlineStr">
         <is>
-          <t>long_term_kalman</t>
+          <t>aggressive</t>
         </is>
       </c>
     </row>
@@ -2685,12 +2698,12 @@
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>HST/MOS</t>
+          <t>STLD/FMC</t>
         </is>
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
-          <t>MOS</t>
+          <t>FMC</t>
         </is>
       </c>
       <c r="D17" s="7" t="inlineStr">
@@ -2699,13 +2712,13 @@
         </is>
       </c>
       <c r="E17" s="24" t="n">
-        <v>-2168</v>
+        <v>-6843</v>
       </c>
       <c r="F17" s="11" t="n">
-        <v>19.82</v>
+        <v>10.8</v>
       </c>
       <c r="G17" s="19" t="n">
-        <v>-42969.76</v>
+        <v>-73904.39999999999</v>
       </c>
       <c r="H17" s="7" t="inlineStr">
         <is>
@@ -2713,11 +2726,11 @@
         </is>
       </c>
       <c r="I17" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J17" s="7" t="inlineStr">
         <is>
-          <t>long_term_kalman</t>
+          <t>aggressive</t>
         </is>
       </c>
     </row>
@@ -2729,12 +2742,12 @@
       </c>
       <c r="B18" s="17" t="inlineStr">
         <is>
-          <t>KLAC/TRMB</t>
+          <t>HST/MOS</t>
         </is>
       </c>
       <c r="C18" s="17" t="inlineStr">
         <is>
-          <t>KLAC</t>
+          <t>HST</t>
         </is>
       </c>
       <c r="D18" s="17" t="inlineStr">
@@ -2743,17 +2756,17 @@
         </is>
       </c>
       <c r="E18" s="26" t="n">
-        <v>470</v>
-      </c>
-      <c r="F18" s="13" t="n">
-        <v>213.56</v>
+        <v>2247</v>
+      </c>
+      <c r="F18" s="15" t="n">
+        <v>23.95</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>100375.08</v>
+        <v>53815.65</v>
       </c>
       <c r="H18" s="17" t="inlineStr">
         <is>
-          <t>tech</t>
+          <t>realestate</t>
         </is>
       </c>
       <c r="I18" s="17" t="n">
@@ -2761,7 +2774,7 @@
       </c>
       <c r="J18" s="17" t="inlineStr">
         <is>
-          <t>monthly_aligned_windows</t>
+          <t>long_term_kalman</t>
         </is>
       </c>
     </row>
@@ -2773,12 +2786,12 @@
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>KLAC/TRMB</t>
+          <t>HST/MOS</t>
         </is>
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>TRMB</t>
+          <t>MOS</t>
         </is>
       </c>
       <c r="D19" s="7" t="inlineStr">
@@ -2787,17 +2800,17 @@
         </is>
       </c>
       <c r="E19" s="24" t="n">
-        <v>-972</v>
+        <v>-2168</v>
       </c>
       <c r="F19" s="11" t="n">
-        <v>50.6</v>
+        <v>19.82</v>
       </c>
       <c r="G19" s="19" t="n">
-        <v>-49183.2</v>
+        <v>-42969.76</v>
       </c>
       <c r="H19" s="7" t="inlineStr">
         <is>
-          <t>industrial</t>
+          <t>food</t>
         </is>
       </c>
       <c r="I19" s="7" t="n">
@@ -2805,7 +2818,7 @@
       </c>
       <c r="J19" s="7" t="inlineStr">
         <is>
-          <t>monthly_aligned_windows</t>
+          <t>long_term_kalman</t>
         </is>
       </c>
     </row>
@@ -2817,12 +2830,12 @@
       </c>
       <c r="B20" s="17" t="inlineStr">
         <is>
-          <t>UNH/ULTA</t>
+          <t>KLAC/TRMB</t>
         </is>
       </c>
       <c r="C20" s="17" t="inlineStr">
         <is>
-          <t>UNH</t>
+          <t>KLAC</t>
         </is>
       </c>
       <c r="D20" s="17" t="inlineStr">
@@ -2831,17 +2844,17 @@
         </is>
       </c>
       <c r="E20" s="26" t="n">
-        <v>124</v>
+        <v>470</v>
       </c>
       <c r="F20" s="13" t="n">
-        <v>407.46</v>
+        <v>213.56</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>50525.04</v>
+        <v>100375.08</v>
       </c>
       <c r="H20" s="17" t="inlineStr">
         <is>
-          <t>health</t>
+          <t>tech</t>
         </is>
       </c>
       <c r="I20" s="17" t="n">
@@ -2849,7 +2862,7 @@
       </c>
       <c r="J20" s="17" t="inlineStr">
         <is>
-          <t>short_term_beta_neutral</t>
+          <t>monthly_aligned_windows</t>
         </is>
       </c>
     </row>
@@ -2861,37 +2874,125 @@
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
+          <t>KLAC/TRMB</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>TRMB</t>
+        </is>
+      </c>
+      <c r="D21" s="7" t="inlineStr">
+        <is>
+          <t>short</t>
+        </is>
+      </c>
+      <c r="E21" s="24" t="n">
+        <v>-972</v>
+      </c>
+      <c r="F21" s="11" t="n">
+        <v>50.6</v>
+      </c>
+      <c r="G21" s="19" t="n">
+        <v>-49183.2</v>
+      </c>
+      <c r="H21" s="7" t="inlineStr">
+        <is>
+          <t>industrial</t>
+        </is>
+      </c>
+      <c r="I21" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J21" s="7" t="inlineStr">
+        <is>
+          <t>monthly_aligned_windows</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="12" t="inlineStr">
+        <is>
+          <t>MTFS</t>
+        </is>
+      </c>
+      <c r="B22" s="17" t="inlineStr">
+        <is>
           <t>UNH/ULTA</t>
         </is>
       </c>
-      <c r="C21" s="7" t="inlineStr">
+      <c r="C22" s="17" t="inlineStr">
+        <is>
+          <t>UNH</t>
+        </is>
+      </c>
+      <c r="D22" s="17" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="E22" s="26" t="n">
+        <v>124</v>
+      </c>
+      <c r="F22" s="13" t="n">
+        <v>407.46</v>
+      </c>
+      <c r="G22" s="13" t="n">
+        <v>50525.04</v>
+      </c>
+      <c r="H22" s="17" t="inlineStr">
+        <is>
+          <t>health</t>
+        </is>
+      </c>
+      <c r="I22" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="J22" s="17" t="inlineStr">
+        <is>
+          <t>short_term_beta_neutral</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="10" t="inlineStr">
+        <is>
+          <t>MTFS</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>UNH/ULTA</t>
+        </is>
+      </c>
+      <c r="C23" s="7" t="inlineStr">
         <is>
           <t>ULTA</t>
         </is>
       </c>
-      <c r="D21" s="7" t="inlineStr">
+      <c r="D23" s="7" t="inlineStr">
         <is>
           <t>short</t>
         </is>
       </c>
-      <c r="E21" s="24" t="n">
+      <c r="E23" s="24" t="n">
         <v>-107</v>
       </c>
-      <c r="F21" s="4" t="n">
+      <c r="F23" s="4" t="n">
         <v>470.75</v>
       </c>
-      <c r="G21" s="19" t="n">
+      <c r="G23" s="19" t="n">
         <v>-50370.25</v>
       </c>
-      <c r="H21" s="7" t="inlineStr">
+      <c r="H23" s="7" t="inlineStr">
         <is>
           <t>food</t>
         </is>
       </c>
-      <c r="I21" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="J21" s="7" t="inlineStr">
+      <c r="I23" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J23" s="7" t="inlineStr">
         <is>
           <t>short_term_beta_neutral</t>
         </is>
@@ -2911,7 +3012,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3001,31 +3102,31 @@
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
         <is>
-          <t>MTFS</t>
+          <t>MRPT</t>
         </is>
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>KLAC/REGN</t>
+          <t>BSX/WMB</t>
         </is>
       </c>
       <c r="C5" s="4" t="n">
-        <v>9083.059999999999</v>
+        <v>1927.19</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>156925.83</v>
+        <v>174184.48</v>
       </c>
       <c r="E5" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>beta_neutral_long_term</t>
+          <t>tight_stop</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">
         <is>
-          <t>long</t>
+          <t>short</t>
         </is>
       </c>
     </row>
@@ -3037,21 +3138,21 @@
       </c>
       <c r="B6" s="17" t="inlineStr">
         <is>
-          <t>NUE/INTU</t>
+          <t>KLAC/REGN</t>
         </is>
       </c>
       <c r="C6" s="13" t="n">
-        <v>4040.63</v>
+        <v>9083.059999999999</v>
       </c>
       <c r="D6" s="13" t="n">
-        <v>105717.25</v>
+        <v>156925.83</v>
       </c>
       <c r="E6" s="17" t="n">
         <v>0</v>
       </c>
       <c r="F6" s="17" t="inlineStr">
         <is>
-          <t>conservative</t>
+          <t>beta_neutral_long_term</t>
         </is>
       </c>
       <c r="G6" s="17" t="inlineStr">
@@ -3068,21 +3169,21 @@
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>NUE/MKTX</t>
+          <t>NUE/INTU</t>
         </is>
       </c>
       <c r="C7" s="4" t="n">
-        <v>6039.67</v>
+        <v>4040.63</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>131409.63</v>
+        <v>105717.25</v>
       </c>
       <c r="E7" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>weekly_aligned_windows</t>
+          <t>conservative</t>
         </is>
       </c>
       <c r="G7" s="7" t="inlineStr">
@@ -3099,21 +3200,21 @@
       </c>
       <c r="B8" s="17" t="inlineStr">
         <is>
-          <t>STLD/UHS</t>
-        </is>
-      </c>
-      <c r="C8" s="35" t="n">
-        <v>-8.06</v>
+          <t>NUE/MKTX</t>
+        </is>
+      </c>
+      <c r="C8" s="13" t="n">
+        <v>6039.67</v>
       </c>
       <c r="D8" s="13" t="n">
-        <v>155424.8</v>
+        <v>131409.63</v>
       </c>
       <c r="E8" s="17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F8" s="17" t="inlineStr">
         <is>
-          <t>no_reversal_protection</t>
+          <t>weekly_aligned_windows</t>
         </is>
       </c>
       <c r="G8" s="17" t="inlineStr">
@@ -3130,21 +3231,21 @@
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>STLD/FMC</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="n">
-        <v>2768.82</v>
+          <t>STLD/UHS</t>
+        </is>
+      </c>
+      <c r="C9" s="35" t="n">
+        <v>-8.06</v>
       </c>
       <c r="D9" s="4" t="n">
-        <v>242421.92</v>
+        <v>155424.8</v>
       </c>
       <c r="E9" s="7" t="n">
         <v>1</v>
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>aggressive</t>
+          <t>no_reversal_protection</t>
         </is>
       </c>
       <c r="G9" s="7" t="inlineStr">
@@ -3161,21 +3262,21 @@
       </c>
       <c r="B10" s="17" t="inlineStr">
         <is>
-          <t>HST/MOS</t>
+          <t>STLD/FMC</t>
         </is>
       </c>
       <c r="C10" s="13" t="n">
-        <v>2281.05</v>
+        <v>2768.82</v>
       </c>
       <c r="D10" s="13" t="n">
-        <v>96785.41</v>
+        <v>242421.92</v>
       </c>
       <c r="E10" s="17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F10" s="17" t="inlineStr">
         <is>
-          <t>long_term_kalman</t>
+          <t>aggressive</t>
         </is>
       </c>
       <c r="G10" s="17" t="inlineStr">
@@ -3192,21 +3293,21 @@
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>KLAC/TRMB</t>
+          <t>HST/MOS</t>
         </is>
       </c>
       <c r="C11" s="4" t="n">
-        <v>2108.89</v>
+        <v>2281.05</v>
       </c>
       <c r="D11" s="4" t="n">
-        <v>149558.28</v>
+        <v>96785.41</v>
       </c>
       <c r="E11" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>monthly_aligned_windows</t>
+          <t>long_term_kalman</t>
         </is>
       </c>
       <c r="G11" s="7" t="inlineStr">
@@ -3223,24 +3324,55 @@
       </c>
       <c r="B12" s="17" t="inlineStr">
         <is>
+          <t>KLAC/TRMB</t>
+        </is>
+      </c>
+      <c r="C12" s="13" t="n">
+        <v>2108.89</v>
+      </c>
+      <c r="D12" s="13" t="n">
+        <v>149558.28</v>
+      </c>
+      <c r="E12" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="17" t="inlineStr">
+        <is>
+          <t>monthly_aligned_windows</t>
+        </is>
+      </c>
+      <c r="G12" s="17" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>MTFS</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
           <t>UNH/ULTA</t>
         </is>
       </c>
-      <c r="C12" s="15" t="n">
+      <c r="C13" s="11" t="n">
         <v>78.09</v>
       </c>
-      <c r="D12" s="13" t="n">
+      <c r="D13" s="4" t="n">
         <v>100895.29</v>
       </c>
-      <c r="E12" s="17" t="n">
-        <v>0</v>
-      </c>
-      <c r="F12" s="17" t="inlineStr">
+      <c r="E13" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="7" t="inlineStr">
         <is>
           <t>short_term_beta_neutral</t>
         </is>
       </c>
-      <c r="G12" s="17" t="inlineStr">
+      <c r="G13" s="7" t="inlineStr">
         <is>
           <t>long</t>
         </is>
@@ -3374,7 +3506,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3534,7 +3666,7 @@
         </is>
       </c>
       <c r="B13" s="7" t="n">
-        <v>26.79</v>
+        <v>24.4</v>
       </c>
     </row>
     <row r="14">
@@ -3544,7 +3676,7 @@
         </is>
       </c>
       <c r="B14" s="17" t="n">
-        <v>23.44</v>
+        <v>22.76</v>
       </c>
     </row>
     <row r="15">
@@ -3554,7 +3686,7 @@
         </is>
       </c>
       <c r="B15" s="7" t="n">
-        <v>16.37</v>
+        <v>15.89</v>
       </c>
     </row>
     <row r="16">
@@ -3564,7 +3696,7 @@
         </is>
       </c>
       <c r="B16" s="17" t="n">
-        <v>10.98</v>
+        <v>11.56</v>
       </c>
     </row>
     <row r="17">
@@ -3574,7 +3706,7 @@
         </is>
       </c>
       <c r="B17" s="7" t="n">
-        <v>8.15</v>
+        <v>8.33</v>
       </c>
     </row>
     <row r="18">
@@ -3584,27 +3716,27 @@
         </is>
       </c>
       <c r="B18" s="17" t="n">
-        <v>7.88</v>
+        <v>7.46</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="10" t="inlineStr">
         <is>
-          <t>HST/MOS</t>
+          <t>BSX/WMB</t>
         </is>
       </c>
       <c r="B19" s="7" t="n">
-        <v>3.65</v>
+        <v>3.58</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="12" t="inlineStr">
         <is>
-          <t>HAS/PFE</t>
+          <t>HST/MOS</t>
         </is>
       </c>
       <c r="B20" s="17" t="n">
-        <v>1.44</v>
+        <v>3.37</v>
       </c>
     </row>
     <row r="21">
@@ -3614,7 +3746,17 @@
         </is>
       </c>
       <c r="B21" s="7" t="n">
-        <v>1.3</v>
+        <v>1.45</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="12" t="inlineStr">
+        <is>
+          <t>HAS/PFE</t>
+        </is>
+      </c>
+      <c r="B22" s="17" t="n">
+        <v>1.18</v>
       </c>
     </row>
   </sheetData>
@@ -4110,7 +4252,7 @@
         <v>1.97</v>
       </c>
       <c r="J9" s="7" t="n">
-        <v>1.243</v>
+        <v>1.409</v>
       </c>
     </row>
     <row r="10">
@@ -4144,7 +4286,7 @@
         <v>2.64</v>
       </c>
       <c r="J10" s="17" t="n">
-        <v>0.304</v>
+        <v>0.612</v>
       </c>
     </row>
     <row r="11">
@@ -4253,7 +4395,7 @@
         </is>
       </c>
       <c r="B5" s="4" t="n">
-        <v>175909.04</v>
+        <v>87801.67</v>
       </c>
       <c r="C5" s="4" t="n">
         <v>136845.07</v>
@@ -4272,7 +4414,7 @@
         </is>
       </c>
       <c r="B6" s="13" t="n">
-        <v>450206.36</v>
+        <v>539796.8100000001</v>
       </c>
       <c r="C6" s="13" t="n">
         <v>500708.01</v>
@@ -4291,7 +4433,7 @@
         </is>
       </c>
       <c r="B7" s="4" t="n">
-        <v>869810.6899999999</v>
+        <v>956161.39</v>
       </c>
       <c r="C7" s="4" t="n">
         <v>909026.52</v>
@@ -4310,7 +4452,7 @@
         </is>
       </c>
       <c r="B8" s="13" t="n">
-        <v>1495926.09</v>
+        <v>1583759.87</v>
       </c>
       <c r="C8" s="13" t="n">
         <v>1546579.6</v>
@@ -4329,7 +4471,7 @@
         </is>
       </c>
       <c r="B9" s="4" t="n">
-        <v>441378.78</v>
+        <v>529212.5600000001</v>
       </c>
       <c r="C9" s="4" t="n">
         <v>490890.21</v>
@@ -4367,7 +4509,7 @@
         </is>
       </c>
       <c r="B11" s="4" t="n">
-        <v>441378.78</v>
+        <v>529212.5600000001</v>
       </c>
       <c r="C11" s="4" t="n">
         <v>490890.21</v>
@@ -4405,7 +4547,7 @@
         </is>
       </c>
       <c r="B13" s="7" t="n">
-        <v>1.243</v>
+        <v>1.409</v>
       </c>
       <c r="C13" s="7" t="n">
         <v>1.326</v>
@@ -4424,7 +4566,7 @@
         </is>
       </c>
       <c r="B14" s="17" t="n">
-        <v>0.406</v>
+        <v>0.405</v>
       </c>
       <c r="C14" s="17" t="n">
         <v>0.396</v>
@@ -4443,7 +4585,7 @@
         </is>
       </c>
       <c r="B15" s="4" t="n">
-        <v>262237.89</v>
+        <v>297074.79</v>
       </c>
       <c r="C15" s="4" t="n">
         <v>279983.35</v>
@@ -4462,7 +4604,7 @@
         </is>
       </c>
       <c r="B16" s="13" t="n">
-        <v>792309.42</v>
+        <v>757472.52</v>
       </c>
       <c r="C16" s="13" t="n">
         <v>775706.04</v>
@@ -4534,7 +4676,7 @@
         </is>
       </c>
       <c r="B21" s="4" t="n">
-        <v>869810.6899999999</v>
+        <v>956161.39</v>
       </c>
       <c r="C21" s="4" t="n">
         <v>909026.52</v>
@@ -4572,7 +4714,7 @@
         </is>
       </c>
       <c r="B23" s="4" t="n">
-        <v>869810.6899999999</v>
+        <v>956161.39</v>
       </c>
       <c r="C23" s="4" t="n">
         <v>909026.52</v>
@@ -4610,7 +4752,7 @@
         </is>
       </c>
       <c r="B25" s="4" t="n">
-        <v>869810.6899999999</v>
+        <v>956161.39</v>
       </c>
       <c r="C25" s="4" t="n">
         <v>909026.52</v>
@@ -4629,7 +4771,7 @@
         </is>
       </c>
       <c r="B26" s="13" t="n">
-        <v>8827.58</v>
+        <v>10584.25</v>
       </c>
       <c r="C26" s="13" t="n">
         <v>9817.799999999999</v>
@@ -4648,7 +4790,7 @@
         </is>
       </c>
       <c r="B27" s="4" t="n">
-        <v>8827.58</v>
+        <v>10584.25</v>
       </c>
       <c r="C27" s="4" t="n">
         <v>9817.799999999999</v>
@@ -4667,7 +4809,7 @@
         </is>
       </c>
       <c r="B28" s="13" t="n">
-        <v>441378.78</v>
+        <v>529212.5600000001</v>
       </c>
       <c r="C28" s="13" t="n">
         <v>490890.21</v>
@@ -4686,7 +4828,7 @@
         </is>
       </c>
       <c r="B29" s="4" t="n">
-        <v>441378.78</v>
+        <v>529212.5600000001</v>
       </c>
       <c r="C29" s="4" t="n">
         <v>490890.21</v>
@@ -4724,7 +4866,7 @@
         </is>
       </c>
       <c r="B31" s="4" t="n">
-        <v>8827.58</v>
+        <v>10584.25</v>
       </c>
       <c r="C31" s="4" t="n">
         <v>9817.799999999999</v>
@@ -4743,7 +4885,7 @@
         </is>
       </c>
       <c r="B32" s="13" t="n">
-        <v>175909.04</v>
+        <v>87801.67</v>
       </c>
       <c r="C32" s="13" t="n">
         <v>136845.07</v>
@@ -4834,7 +4976,7 @@
         </is>
       </c>
       <c r="B39" s="4" t="n">
-        <v>478787.36</v>
+        <v>390679.98</v>
       </c>
       <c r="C39" s="4" t="n">
         <v>468937.27</v>
@@ -4853,7 +4995,7 @@
         </is>
       </c>
       <c r="B40" s="13" t="n">
-        <v>88702.46000000001</v>
+        <v>178292.92</v>
       </c>
       <c r="C40" s="13" t="n">
         <v>99198.59</v>
@@ -4872,7 +5014,7 @@
         </is>
       </c>
       <c r="B41" s="4" t="n">
-        <v>85087.86</v>
+        <v>171438.56</v>
       </c>
       <c r="C41" s="4" t="n">
         <v>96238.08</v>
@@ -4891,7 +5033,7 @@
         </is>
       </c>
       <c r="B42" s="13" t="n">
-        <v>652577.6800000001</v>
+        <v>740411.46</v>
       </c>
       <c r="C42" s="13" t="n">
         <v>664373.9399999999</v>
@@ -4910,7 +5052,7 @@
         </is>
       </c>
       <c r="B43" s="4" t="n">
-        <v>86963.2</v>
+        <v>174796.98</v>
       </c>
       <c r="C43" s="4" t="n">
         <v>97253.52</v>
@@ -4948,7 +5090,7 @@
         </is>
       </c>
       <c r="B45" s="4" t="n">
-        <v>86963.2</v>
+        <v>174796.98</v>
       </c>
       <c r="C45" s="4" t="n">
         <v>97253.52</v>
@@ -4986,7 +5128,7 @@
         </is>
       </c>
       <c r="B47" s="7" t="n">
-        <v>0.304</v>
+        <v>0.612</v>
       </c>
       <c r="C47" s="7" t="n">
         <v>0.341</v>
@@ -5005,7 +5147,7 @@
         </is>
       </c>
       <c r="B48" s="17" t="n">
-        <v>-0.003</v>
+        <v>-0.006</v>
       </c>
       <c r="C48" s="17" t="n">
         <v>-0.002</v>
@@ -5024,7 +5166,7 @@
         </is>
       </c>
       <c r="B49" s="4" t="n">
-        <v>34410.21</v>
+        <v>69247.11</v>
       </c>
       <c r="C49" s="4" t="n">
         <v>38698.32</v>
@@ -5043,7 +5185,7 @@
         </is>
       </c>
       <c r="B50" s="13" t="n">
-        <v>531204.27</v>
+        <v>496367.37</v>
       </c>
       <c r="C50" s="13" t="n">
         <v>528422.1</v>
@@ -5115,7 +5257,7 @@
         </is>
       </c>
       <c r="B55" s="4" t="n">
-        <v>85087.86</v>
+        <v>171438.56</v>
       </c>
       <c r="C55" s="4" t="n">
         <v>96238.08</v>
@@ -5153,7 +5295,7 @@
         </is>
       </c>
       <c r="B57" s="4" t="n">
-        <v>85087.86</v>
+        <v>171438.56</v>
       </c>
       <c r="C57" s="4" t="n">
         <v>96238.08</v>
@@ -5191,7 +5333,7 @@
         </is>
       </c>
       <c r="B59" s="4" t="n">
-        <v>85087.86</v>
+        <v>171438.56</v>
       </c>
       <c r="C59" s="4" t="n">
         <v>96238.08</v>
@@ -5210,7 +5352,7 @@
         </is>
       </c>
       <c r="B60" s="13" t="n">
-        <v>1739.26</v>
+        <v>3495.94</v>
       </c>
       <c r="C60" s="13" t="n">
         <v>1945.07</v>
@@ -5229,7 +5371,7 @@
         </is>
       </c>
       <c r="B61" s="4" t="n">
-        <v>1739.26</v>
+        <v>3495.94</v>
       </c>
       <c r="C61" s="4" t="n">
         <v>1945.07</v>
@@ -5248,7 +5390,7 @@
         </is>
       </c>
       <c r="B62" s="13" t="n">
-        <v>86963.2</v>
+        <v>174796.98</v>
       </c>
       <c r="C62" s="13" t="n">
         <v>97253.52</v>
@@ -5267,7 +5409,7 @@
         </is>
       </c>
       <c r="B63" s="4" t="n">
-        <v>86963.2</v>
+        <v>174796.98</v>
       </c>
       <c r="C63" s="4" t="n">
         <v>97253.52</v>
@@ -5305,7 +5447,7 @@
         </is>
       </c>
       <c r="B65" s="4" t="n">
-        <v>1739.26</v>
+        <v>3495.94</v>
       </c>
       <c r="C65" s="4" t="n">
         <v>1945.07</v>
@@ -5324,7 +5466,7 @@
         </is>
       </c>
       <c r="B66" s="13" t="n">
-        <v>478787.36</v>
+        <v>390679.98</v>
       </c>
       <c r="C66" s="13" t="n">
         <v>468937.27</v>
@@ -6065,7 +6207,7 @@
         </is>
       </c>
       <c r="B7" s="4" t="n">
-        <v>24694.87</v>
+        <v>26622.06</v>
       </c>
     </row>
     <row r="9">
@@ -6146,8 +6288,8 @@
           <t>Current unrealized PnL</t>
         </is>
       </c>
-      <c r="B13" s="19" t="n">
-        <v>-1697.28</v>
+      <c r="B13" s="4" t="n">
+        <v>229.91</v>
       </c>
     </row>
     <row r="15">
@@ -6828,7 +6970,7 @@
         </is>
       </c>
       <c r="B5" s="4" t="n">
-        <v>616536.01</v>
+        <v>618019.09</v>
       </c>
     </row>
     <row r="6">
@@ -6848,7 +6990,7 @@
         </is>
       </c>
       <c r="B7" s="19" t="n">
-        <v>-373379.97</v>
+        <v>-371896.89</v>
       </c>
     </row>
     <row r="8">
@@ -6868,7 +7010,7 @@
         </is>
       </c>
       <c r="B9" s="4" t="n">
-        <v>175909.04</v>
+        <v>87801.67</v>
       </c>
     </row>
     <row r="11">
@@ -8543,31 +8685,31 @@
         <v>1054547.31</v>
       </c>
       <c r="C4" s="4" t="n">
-        <v>869810.6899999999</v>
+        <v>956161.39</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>441378.78</v>
+        <v>529212.5600000001</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>1311189.47</v>
+        <v>1485373.95</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>428431.91</v>
+        <v>426948.83</v>
       </c>
       <c r="G4" s="5" t="n">
-        <v>1.243</v>
+        <v>1.409</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>0.406</v>
+        <v>0.405</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>124.34</v>
+        <v>140.85</v>
       </c>
       <c r="J4" s="5" t="n">
-        <v>62.17</v>
+        <v>70.43000000000001</v>
       </c>
       <c r="K4" s="24" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5">
@@ -8580,31 +8722,31 @@
         <v>565614.48</v>
       </c>
       <c r="C5" s="13" t="n">
-        <v>85087.86</v>
+        <v>171438.56</v>
       </c>
       <c r="D5" s="13" t="n">
-        <v>86963.2</v>
+        <v>174796.98</v>
       </c>
       <c r="E5" s="13" t="n">
-        <v>172051.06</v>
+        <v>346235.54</v>
       </c>
       <c r="F5" s="18" t="n">
-        <v>-1875.34</v>
+        <v>-3358.42</v>
       </c>
       <c r="G5" s="25" t="n">
-        <v>0.304</v>
+        <v>0.612</v>
       </c>
       <c r="H5" s="25" t="n">
-        <v>-0.003</v>
+        <v>-0.006</v>
       </c>
       <c r="I5" s="25" t="n">
-        <v>30.42</v>
+        <v>61.21</v>
       </c>
       <c r="J5" s="25" t="n">
-        <v>15.21</v>
+        <v>30.61</v>
       </c>
       <c r="K5" s="26" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6">
@@ -8658,7 +8800,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F25"/>
+  <dimension ref="A1:F26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -8679,7 +8821,7 @@
     <row r="3">
       <c r="A3" s="27" t="inlineStr">
         <is>
-          <t>HHI=0.1207  ·  effective N pairs=8.3  ·  max pair=18.49% of gross</t>
+          <t>HHI=0.1078  ·  effective N pairs=9.3  ·  max pair=16.32% of gross</t>
         </is>
       </c>
     </row>
@@ -8731,7 +8873,7 @@
         <v>25.8</v>
       </c>
       <c r="E6" s="23" t="n">
-        <v>20.75</v>
+        <v>18.32</v>
       </c>
       <c r="F6" s="24" t="n">
         <v>2</v>
@@ -8753,7 +8895,7 @@
         <v>23.09</v>
       </c>
       <c r="E7" s="21" t="n">
-        <v>18.57</v>
+        <v>16.39</v>
       </c>
       <c r="F7" s="26" t="n">
         <v>2</v>
@@ -8775,7 +8917,7 @@
         <v>15.63</v>
       </c>
       <c r="E8" s="23" t="n">
-        <v>12.57</v>
+        <v>11.1</v>
       </c>
       <c r="F8" s="24" t="n">
         <v>2</v>
@@ -8784,20 +8926,20 @@
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
         <is>
-          <t>PFE</t>
+          <t>BSX</t>
         </is>
       </c>
       <c r="B9" s="13" t="n">
-        <v>86963.2</v>
+        <v>87833.78</v>
       </c>
       <c r="C9" s="18" t="n">
-        <v>-86963.2</v>
+        <v>-87833.78</v>
       </c>
       <c r="D9" s="21" t="n">
-        <v>8.25</v>
+        <v>8.33</v>
       </c>
       <c r="E9" s="21" t="n">
-        <v>6.63</v>
+        <v>5.91</v>
       </c>
       <c r="F9" s="26" t="n">
         <v>1</v>
@@ -8806,20 +8948,20 @@
     <row r="10">
       <c r="A10" s="10" t="inlineStr">
         <is>
-          <t>HAS</t>
+          <t>PFE</t>
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>85087.86</v>
-      </c>
-      <c r="C10" s="4" t="n">
-        <v>85087.86</v>
+        <v>86963.2</v>
+      </c>
+      <c r="C10" s="19" t="n">
+        <v>-86963.2</v>
       </c>
       <c r="D10" s="23" t="n">
-        <v>8.07</v>
+        <v>8.25</v>
       </c>
       <c r="E10" s="23" t="n">
-        <v>6.49</v>
+        <v>5.85</v>
       </c>
       <c r="F10" s="24" t="n">
         <v>1</v>
@@ -8828,20 +8970,20 @@
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
         <is>
-          <t>FMC</t>
+          <t>WMB</t>
         </is>
       </c>
       <c r="B11" s="13" t="n">
-        <v>73904.39999999999</v>
-      </c>
-      <c r="C11" s="18" t="n">
-        <v>-73904.39999999999</v>
+        <v>86350.7</v>
+      </c>
+      <c r="C11" s="13" t="n">
+        <v>86350.7</v>
       </c>
       <c r="D11" s="21" t="n">
-        <v>7.01</v>
+        <v>8.19</v>
       </c>
       <c r="E11" s="21" t="n">
-        <v>5.64</v>
+        <v>5.81</v>
       </c>
       <c r="F11" s="26" t="n">
         <v>1</v>
@@ -8850,20 +8992,20 @@
     <row r="12">
       <c r="A12" s="10" t="inlineStr">
         <is>
-          <t>HST</t>
+          <t>HAS</t>
         </is>
       </c>
       <c r="B12" s="4" t="n">
-        <v>53815.65</v>
+        <v>85087.86</v>
       </c>
       <c r="C12" s="4" t="n">
-        <v>53815.65</v>
+        <v>85087.86</v>
       </c>
       <c r="D12" s="23" t="n">
-        <v>5.1</v>
+        <v>8.07</v>
       </c>
       <c r="E12" s="23" t="n">
-        <v>4.1</v>
+        <v>5.73</v>
       </c>
       <c r="F12" s="24" t="n">
         <v>1</v>
@@ -8872,20 +9014,20 @@
     <row r="13">
       <c r="A13" s="12" t="inlineStr">
         <is>
-          <t>UHS</t>
+          <t>FMC</t>
         </is>
       </c>
       <c r="B13" s="13" t="n">
-        <v>51845.56</v>
+        <v>73904.39999999999</v>
       </c>
       <c r="C13" s="18" t="n">
-        <v>-51845.56</v>
+        <v>-73904.39999999999</v>
       </c>
       <c r="D13" s="21" t="n">
-        <v>4.92</v>
+        <v>7.01</v>
       </c>
       <c r="E13" s="21" t="n">
-        <v>3.95</v>
+        <v>4.98</v>
       </c>
       <c r="F13" s="26" t="n">
         <v>1</v>
@@ -8894,20 +9036,20 @@
     <row r="14">
       <c r="A14" s="10" t="inlineStr">
         <is>
-          <t>UNH</t>
+          <t>HST</t>
         </is>
       </c>
       <c r="B14" s="4" t="n">
-        <v>50525.04</v>
+        <v>53815.65</v>
       </c>
       <c r="C14" s="4" t="n">
-        <v>50525.04</v>
+        <v>53815.65</v>
       </c>
       <c r="D14" s="23" t="n">
-        <v>4.79</v>
+        <v>5.1</v>
       </c>
       <c r="E14" s="23" t="n">
-        <v>3.85</v>
+        <v>3.62</v>
       </c>
       <c r="F14" s="24" t="n">
         <v>1</v>
@@ -8916,20 +9058,20 @@
     <row r="15">
       <c r="A15" s="12" t="inlineStr">
         <is>
-          <t>ULTA</t>
+          <t>UHS</t>
         </is>
       </c>
       <c r="B15" s="13" t="n">
-        <v>50370.25</v>
+        <v>51845.56</v>
       </c>
       <c r="C15" s="18" t="n">
-        <v>-50370.25</v>
+        <v>-51845.56</v>
       </c>
       <c r="D15" s="21" t="n">
-        <v>4.78</v>
+        <v>4.92</v>
       </c>
       <c r="E15" s="21" t="n">
-        <v>3.84</v>
+        <v>3.49</v>
       </c>
       <c r="F15" s="26" t="n">
         <v>1</v>
@@ -8985,102 +9127,121 @@
         <v>436919.18</v>
       </c>
       <c r="E20" s="7" t="n">
-        <v>33.32</v>
+        <v>29.41</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="12" t="inlineStr">
         <is>
-          <t>tech</t>
+          <t>health</t>
         </is>
       </c>
       <c r="B21" s="13" t="n">
-        <v>243462.96</v>
+        <v>50525.04</v>
       </c>
       <c r="C21" s="13" t="n">
-        <v>72304.46000000001</v>
-      </c>
-      <c r="D21" s="13" t="n">
-        <v>171158.5</v>
+        <v>240480.49</v>
+      </c>
+      <c r="D21" s="18" t="n">
+        <v>-189955.45</v>
       </c>
       <c r="E21" s="17" t="n">
-        <v>13.05</v>
+        <v>-12.79</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="10" t="inlineStr">
         <is>
-          <t>health</t>
+          <t>tech</t>
         </is>
       </c>
       <c r="B22" s="4" t="n">
-        <v>50525.04</v>
+        <v>243462.96</v>
       </c>
       <c r="C22" s="4" t="n">
-        <v>152646.71</v>
-      </c>
-      <c r="D22" s="19" t="n">
-        <v>-102121.67</v>
+        <v>72304.46000000001</v>
+      </c>
+      <c r="D22" s="4" t="n">
+        <v>171158.5</v>
       </c>
       <c r="E22" s="7" t="n">
-        <v>-7.79</v>
+        <v>11.52</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="12" t="inlineStr">
         <is>
-          <t>food</t>
+          <t>energy</t>
         </is>
       </c>
       <c r="B23" s="13" t="n">
-        <v>85087.86</v>
-      </c>
-      <c r="C23" s="13" t="n">
-        <v>167244.41</v>
-      </c>
-      <c r="D23" s="18" t="n">
-        <v>-82156.55</v>
+        <v>86350.7</v>
+      </c>
+      <c r="C23" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="D23" s="13" t="n">
+        <v>86350.7</v>
       </c>
       <c r="E23" s="17" t="n">
-        <v>-6.27</v>
+        <v>5.81</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="10" t="inlineStr">
         <is>
-          <t>realestate</t>
+          <t>food</t>
         </is>
       </c>
       <c r="B24" s="4" t="n">
-        <v>53815.65</v>
-      </c>
-      <c r="C24" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="D24" s="4" t="n">
-        <v>53815.65</v>
+        <v>85087.86</v>
+      </c>
+      <c r="C24" s="4" t="n">
+        <v>167244.41</v>
+      </c>
+      <c r="D24" s="19" t="n">
+        <v>-82156.55</v>
       </c>
       <c r="E24" s="7" t="n">
-        <v>4.1</v>
+        <v>-5.53</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="12" t="inlineStr">
         <is>
+          <t>realestate</t>
+        </is>
+      </c>
+      <c r="B25" s="13" t="n">
+        <v>53815.65</v>
+      </c>
+      <c r="C25" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="D25" s="13" t="n">
+        <v>53815.65</v>
+      </c>
+      <c r="E25" s="17" t="n">
+        <v>3.62</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="10" t="inlineStr">
+        <is>
           <t>industrial</t>
         </is>
       </c>
-      <c r="B25" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="C25" s="13" t="n">
+      <c r="B26" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="4" t="n">
         <v>49183.2</v>
       </c>
-      <c r="D25" s="18" t="n">
+      <c r="D26" s="19" t="n">
         <v>-49183.2</v>
       </c>
-      <c r="E25" s="17" t="n">
-        <v>-3.75</v>
+      <c r="E26" s="7" t="n">
+        <v>-3.31</v>
       </c>
     </row>
   </sheetData>
@@ -9097,7 +9258,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -9118,7 +9279,7 @@
         </is>
       </c>
       <c r="B3" s="6" t="n">
-        <v>0.804</v>
+        <v>0.768</v>
       </c>
     </row>
     <row r="4">
@@ -9128,7 +9289,7 @@
         </is>
       </c>
       <c r="B4" s="5" t="n">
-        <v>1.284</v>
+        <v>1.32</v>
       </c>
     </row>
     <row r="5">
@@ -9179,57 +9340,67 @@
         </is>
       </c>
       <c r="B10" s="23" t="n">
-        <v>33.32</v>
+        <v>29.41</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
         <is>
-          <t>tech</t>
-        </is>
-      </c>
-      <c r="B11" s="21" t="n">
-        <v>13.05</v>
+          <t>health</t>
+        </is>
+      </c>
+      <c r="B11" s="20" t="n">
+        <v>-12.79</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="10" t="inlineStr">
         <is>
-          <t>health</t>
-        </is>
-      </c>
-      <c r="B12" s="22" t="n">
-        <v>-7.79</v>
+          <t>tech</t>
+        </is>
+      </c>
+      <c r="B12" s="23" t="n">
+        <v>11.52</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="12" t="inlineStr">
         <is>
-          <t>food</t>
-        </is>
-      </c>
-      <c r="B13" s="20" t="n">
-        <v>-6.27</v>
+          <t>energy</t>
+        </is>
+      </c>
+      <c r="B13" s="21" t="n">
+        <v>5.81</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="10" t="inlineStr">
         <is>
-          <t>realestate</t>
-        </is>
-      </c>
-      <c r="B14" s="23" t="n">
-        <v>4.1</v>
+          <t>food</t>
+        </is>
+      </c>
+      <c r="B14" s="22" t="n">
+        <v>-5.53</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">
         <is>
+          <t>realestate</t>
+        </is>
+      </c>
+      <c r="B15" s="21" t="n">
+        <v>3.62</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="10" t="inlineStr">
+        <is>
           <t>industrial</t>
         </is>
       </c>
-      <c r="B15" s="20" t="n">
-        <v>-3.75</v>
+      <c r="B16" s="22" t="n">
+        <v>-3.31</v>
       </c>
     </row>
   </sheetData>

</xml_diff>